<commit_message>
Kahoot: numeric time-limit and correct-answer cells, plus template mode
Columns F and G are written as numbers again; A-E stay strings. The
importer had rejected string-formatted numbers there.

Because a reconstructed header row is still a guess, the script can now
open Kahoot's own downloaded template (kahoot/template.xlsx, gitignored),
write the question rows into it from row 9 down, and leave every other
part of their file byte-identical. That needs real zip inflate/deflate,
so the writer now handles both.

Generation also validates before writing and fails loudly: question <= 120
chars, answers <= 75, time limit from the allowed set, correct answer 1-4
pointing at a non-empty answer. All 104 questions pass, with the longest
question at 112 and the longest answer at 58.
</commit_message>
<xml_diff>
--- a/kahoot/week01.xlsx
+++ b/kahoot/week01.xlsx
@@ -14,7 +14,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kahoot! quiz — question import</t>
+          <t xml:space="preserve">Kahoot! quiz - question import</t>
         </is>
       </c>
     </row>
@@ -105,15 +105,11 @@
           <t xml:space="preserve">Let n be a natural number</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3</t>
-        </is>
+      <c r="F9">
+        <v>30</v>
+      </c>
+      <c r="G9">
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -142,15 +138,11 @@
           <t xml:space="preserve">depends on the meaning of A</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
+      <c r="F10">
+        <v>20</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -179,15 +171,11 @@
           <t xml:space="preserve">3</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2</t>
-        </is>
+      <c r="F11">
+        <v>20</v>
+      </c>
+      <c r="G11">
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -216,15 +204,11 @@
           <t xml:space="preserve">A xor B</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2</t>
-        </is>
+      <c r="F12">
+        <v>30</v>
+      </c>
+      <c r="G12">
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -253,15 +237,11 @@
           <t xml:space="preserve">A implies B</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3</t>
-        </is>
+      <c r="F13">
+        <v>30</v>
+      </c>
+      <c r="G13">
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -290,15 +270,11 @@
           <t xml:space="preserve">induction was needed</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2</t>
-        </is>
+      <c r="F14">
+        <v>30</v>
+      </c>
+      <c r="G14">
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -327,15 +303,11 @@
           <t xml:space="preserve">24</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">60</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3</t>
-        </is>
+      <c r="F15">
+        <v>60</v>
+      </c>
+      <c r="G15">
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -364,15 +336,11 @@
           <t xml:space="preserve">idempotence</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3</t>
-        </is>
+      <c r="F16">
+        <v>30</v>
+      </c>
+      <c r="G16">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>